<commit_message>
feat: Retailer Marking, Activation Report, and UI enhancements
</commit_message>
<xml_diff>
--- a/backend/_data_list/FF_Master.xlsx
+++ b/backend/_data_list/FF_Master.xlsx
@@ -5,18 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\OrangeFlow_Dev\_data_list\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04\home\neelima\projects\Orange-Flow-Next-Js\backend\_data_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87194FEE-4304-40C6-A51A-151B25E1344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCACB50-8869-4B73-8DDD-339E585DC8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AK$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="315">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -981,6 +984,9 @@
   </si>
   <si>
     <t>Tanvir</t>
+  </si>
+  <si>
+    <t>USERNAME</t>
   </si>
 </sst>
 </file>
@@ -1039,20 +1045,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1076,6 +1070,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1113,6 +1128,191 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="B1" t="str">
+            <v>NAME</v>
+          </cell>
+          <cell r="C1" t="str">
+            <v>USERNAME</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="B2" t="str">
+            <v>Shamsuzzaman Patwary</v>
+          </cell>
+          <cell r="C2" t="str">
+            <v>spatwary</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="B3" t="str">
+            <v>Khasruzzaman Khasru</v>
+          </cell>
+          <cell r="C3" t="str">
+            <v>khasruzzaman</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="B4" t="str">
+            <v>Titu Mia</v>
+          </cell>
+          <cell r="C4" t="str">
+            <v>titumia</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="B5" t="str">
+            <v>Toriqul Islam</v>
+          </cell>
+          <cell r="C5" t="str">
+            <v>toriqulislam</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="B6" t="str">
+            <v>Sher Ali</v>
+          </cell>
+          <cell r="C6" t="str">
+            <v>sherali</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="B7" t="str">
+            <v>Md. Ali Hossein</v>
+          </cell>
+          <cell r="C7" t="str">
+            <v>alihossein</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="B8" t="str">
+            <v>Mijan</v>
+          </cell>
+          <cell r="C8" t="str">
+            <v>mijan</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="B9" t="str">
+            <v>Mahmud Hasan Emon</v>
+          </cell>
+          <cell r="C9" t="str">
+            <v>mahmudhasan</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="B10" t="str">
+            <v>Saddam</v>
+          </cell>
+          <cell r="C10" t="str">
+            <v>saddam</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="B11" t="str">
+            <v>Tanvir Patwary</v>
+          </cell>
+          <cell r="C11" t="str">
+            <v>tanvirpatwary</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="B12" t="str">
+            <v>Mahammudul Hasan Shuva</v>
+          </cell>
+          <cell r="C12" t="str">
+            <v>mahammudulhasan</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="B13" t="str">
+            <v>Safiqul Islam</v>
+          </cell>
+          <cell r="C13" t="str">
+            <v>safiqulislam</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="B14" t="str">
+            <v>Md. Hasan Mia</v>
+          </cell>
+          <cell r="C14" t="str">
+            <v>hasanmia</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="B15" t="str">
+            <v>Kaiyum Mia</v>
+          </cell>
+          <cell r="C15" t="str">
+            <v>kaiyummia</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="B16" t="str">
+            <v>Feroz Mia</v>
+          </cell>
+          <cell r="C16" t="str">
+            <v>ferozmia</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="B17" t="str">
+            <v>Hridoy Mia</v>
+          </cell>
+          <cell r="C17" t="str">
+            <v>hridoymia365</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="B18" t="str">
+            <v>Siam Talukdar</v>
+          </cell>
+          <cell r="C18" t="str">
+            <v>siamtalukdar</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="B19" t="str">
+            <v>Md. Hridoy Mia</v>
+          </cell>
+          <cell r="C19" t="str">
+            <v>hridoymia366</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="B20" t="str">
+            <v>Shuvo</v>
+          </cell>
+          <cell r="C20" t="str">
+            <v>shuvo</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="B21" t="str">
+            <v>Sabbir Ahmed Bappy</v>
+          </cell>
+          <cell r="C21" t="str">
+            <v>sabbirahmed</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1400,2849 +1600,2914 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AK43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AL43"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" style="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29" style="13" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14" style="13" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10" style="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.28515625" style="15" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.5703125" style="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.7109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="41.7109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="44.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="35.7109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="38.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="27" style="13" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="53.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="32.140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="33.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="17.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.5703125" style="13" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="12.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="13"/>
+    <col min="1" max="1" width="11.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14" style="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="41.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="44.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="35.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="38.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="29" max="30" width="27" style="5" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="53.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="32.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="33.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="17.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="21.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="39" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="M1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="N1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="P1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="Q1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="R1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="S1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="T1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="U1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="V1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="W1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="X1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="Y1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Z1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="AA1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AA1" s="9" t="s">
+      <c r="AB1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AB1" s="9" t="s">
+      <c r="AC1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AC1" s="9" t="s">
+      <c r="AD1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AF1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AF1" s="9" t="s">
+      <c r="AG1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AG1" s="9" t="s">
+      <c r="AH1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AH1" s="9" t="s">
+      <c r="AI1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AI1" s="9" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AJ1" s="9" t="s">
+      <c r="AK1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AK1" s="9" t="s">
+      <c r="AL1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>alihossein</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="9">
         <v>1409944001</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="9">
         <v>1831949395</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="9">
         <v>1935593311</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="1">
+      <c r="K2" s="9">
         <v>8000</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L2" s="2">
+      <c r="M2" s="10">
         <v>45505</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="1" t="s">
+      <c r="N2" s="10"/>
+      <c r="O2" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O2" s="2">
+      <c r="P2" s="10">
         <v>37174</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="R2" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R2" s="3">
+      <c r="S2" s="11">
         <v>1731580054121</v>
       </c>
-      <c r="AK2" s="1" t="s">
+      <c r="AL2" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>safiqulislam</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="1">
+      <c r="G3" s="9">
         <v>1409944003</v>
       </c>
-      <c r="G3" s="1">
+      <c r="H3" s="9">
         <v>1642536878</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="9">
         <v>1935593312</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J3" s="1">
+      <c r="K3" s="9">
         <v>7350</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L3" s="2">
+      <c r="M3" s="10">
         <v>44896</v>
       </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="10"/>
+      <c r="O3" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O3" s="2">
+      <c r="P3" s="10">
         <v>36392</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="Q3" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="R3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R3" s="3">
+      <c r="S3" s="11">
         <v>1731580028841</v>
       </c>
-      <c r="AK3" s="1" t="s">
+      <c r="AL3" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>saddam</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="9">
         <v>1908441954</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="9">
         <v>1911916176</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="9">
         <v>1935591829</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="J4" s="1">
+      <c r="K4" s="9">
         <v>9260</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L4" s="2">
+      <c r="M4" s="10">
         <v>43132</v>
       </c>
-      <c r="M4" s="2"/>
-      <c r="N4" s="1" t="s">
+      <c r="N4" s="10"/>
+      <c r="O4" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O4" s="2">
+      <c r="P4" s="10">
         <v>34856</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="Q4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="R4" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R4" s="3">
+      <c r="S4" s="11">
         <v>1731030011186</v>
       </c>
-      <c r="AK4" s="1" t="s">
+      <c r="AL4" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="1">
+      <c r="G5" s="9">
         <v>1908441955</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="9">
         <v>1935591837</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="J5" s="1">
+      <c r="K5" s="9">
         <v>9662</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L5" s="2">
+      <c r="M5" s="10">
         <v>43160</v>
       </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="1" t="s">
+      <c r="N5" s="10"/>
+      <c r="O5" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O5" s="2">
+      <c r="P5" s="10">
         <v>29571</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="Q5" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="R5" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R5" s="3">
+      <c r="S5" s="11">
         <v>1731510158618</v>
       </c>
-      <c r="AK5" s="1" t="s">
+      <c r="AL5" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="1">
+      <c r="G6" s="9">
         <v>1915270101</v>
       </c>
-      <c r="H6" s="1">
+      <c r="I6" s="9">
         <v>1935591856</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="J6" s="1">
+      <c r="K6" s="9">
         <v>8349</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L6" s="2">
+      <c r="M6" s="10">
         <v>43525</v>
       </c>
-      <c r="M6" s="2"/>
-      <c r="N6" s="1" t="s">
+      <c r="N6" s="10"/>
+      <c r="O6" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O6" s="2">
+      <c r="P6" s="10">
         <v>37235</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="Q6" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="R6" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="R6" s="3">
+      <c r="S6" s="11">
         <v>7017512906614</v>
       </c>
-      <c r="AK6" s="1" t="s">
+      <c r="AL6" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="1">
+      <c r="G7" s="9">
         <v>1915270102</v>
       </c>
-      <c r="H7" s="1">
+      <c r="I7" s="9">
         <v>1935592000</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="J7" s="1">
+      <c r="K7" s="9">
         <v>8500</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="L7" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L7" s="2">
+      <c r="M7" s="10">
         <v>45840</v>
       </c>
-      <c r="M7" s="2"/>
-      <c r="N7" s="1" t="s">
+      <c r="N7" s="10"/>
+      <c r="O7" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O7" s="2">
+      <c r="P7" s="10">
         <v>38178</v>
       </c>
-      <c r="P7" s="1" t="s">
+      <c r="Q7" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="Q7" s="1" t="s">
+      <c r="R7" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R7" s="3">
+      <c r="S7" s="11">
         <v>1731580357541</v>
       </c>
-      <c r="AK7" s="1" t="s">
+      <c r="AL7" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>mahammudulhasan</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="1">
+      <c r="G8" s="9">
         <v>1915270103</v>
       </c>
-      <c r="G8" s="1">
+      <c r="H8" s="9">
         <v>1813862410</v>
       </c>
-      <c r="H8" s="1">
+      <c r="I8" s="9">
         <v>1935591914</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="J8" s="1">
+      <c r="K8" s="9">
         <v>8500</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="L8" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L8" s="2">
+      <c r="M8" s="10">
         <v>46062</v>
       </c>
-      <c r="M8" s="2">
+      <c r="N8" s="10">
         <v>46142</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="O8" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O8" s="2">
+      <c r="P8" s="10">
         <v>38716</v>
       </c>
-      <c r="P8" s="1" t="s">
+      <c r="Q8" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="Q8" s="1" t="s">
+      <c r="R8" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="R8" s="3">
+      <c r="S8" s="11">
         <v>2311030477929</v>
       </c>
-      <c r="AK8" s="1" t="s">
+      <c r="AL8" s="9" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:37" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:38" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="F9" s="4">
+      <c r="G9" s="12">
         <v>1915270103</v>
       </c>
-      <c r="G9" s="4">
+      <c r="H9" s="12">
         <v>1764864677</v>
       </c>
-      <c r="H9" s="4">
+      <c r="I9" s="12">
         <v>1935591914</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="J9" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="J9" s="4">
+      <c r="K9" s="12">
         <v>9500</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="L9" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="L9" s="5">
+      <c r="M9" s="13">
         <v>46143</v>
       </c>
-      <c r="M9" s="5"/>
-      <c r="N9" s="4" t="s">
+      <c r="N9" s="13"/>
+      <c r="O9" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="O9" s="5">
+      <c r="P9" s="13">
         <v>38512</v>
       </c>
-      <c r="P9" s="6">
+      <c r="Q9" s="8">
         <v>7824872522</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="R9" s="8">
+      <c r="S9" s="15">
         <v>2311030553506</v>
       </c>
-      <c r="U9" s="4" t="s">
+      <c r="V9" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="V9" s="4" t="s">
+      <c r="W9" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="W9" s="4">
+      <c r="X9" s="12">
         <v>1742609199</v>
       </c>
-      <c r="X9" s="4" t="s">
+      <c r="Y9" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="Y9" s="4" t="s">
+      <c r="Z9" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="Z9" s="4" t="s">
+      <c r="AA9" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="AA9" s="4" t="s">
+      <c r="AB9" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AB9" s="4" t="s">
+      <c r="AC9" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="AC9" s="4" t="s">
+      <c r="AD9" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="AD9" s="4" t="s">
+      <c r="AE9" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="AE9" s="4" t="s">
+      <c r="AF9" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="AF9" s="4" t="s">
+      <c r="AG9" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="AG9" s="4">
+      <c r="AH9" s="12">
         <v>9000</v>
       </c>
-      <c r="AH9" s="4" t="s">
+      <c r="AI9" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="AI9" s="4" t="s">
+      <c r="AJ9" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="AJ9" s="4" t="s">
+      <c r="AK9" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="AK9" s="4" t="s">
+      <c r="AL9" s="12" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="1">
+      <c r="G10" s="9">
         <v>1915270106</v>
       </c>
-      <c r="H10" s="1">
+      <c r="I10" s="9">
         <v>1935591815</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="J10" s="1">
+      <c r="K10" s="9">
         <v>8500</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="L10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L10" s="2">
+      <c r="M10" s="10">
         <v>45909</v>
       </c>
-      <c r="M10" s="2"/>
-      <c r="N10" s="1" t="s">
+      <c r="N10" s="10"/>
+      <c r="O10" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O10" s="2">
+      <c r="P10" s="10">
         <v>37448</v>
       </c>
-      <c r="P10" s="1" t="s">
+      <c r="Q10" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="Q10" s="1" t="s">
+      <c r="R10" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R10" s="3">
+      <c r="S10" s="11">
         <v>2311030377356</v>
       </c>
-      <c r="AK10" s="1" t="s">
+      <c r="AL10" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>kaiyummia</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="1">
+      <c r="G11" s="9">
         <v>1915300196</v>
       </c>
-      <c r="G11" s="1">
+      <c r="H11" s="9">
         <v>1917509966</v>
       </c>
-      <c r="H11" s="1">
+      <c r="I11" s="9">
         <v>1935591797</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="J11" s="1">
+      <c r="K11" s="9">
         <v>8500</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="L11" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L11" s="2">
+      <c r="M11" s="10">
         <v>45873</v>
       </c>
-      <c r="M11" s="2"/>
-      <c r="N11" s="1" t="s">
+      <c r="N11" s="10"/>
+      <c r="O11" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O11" s="2">
+      <c r="P11" s="10">
         <v>36526</v>
       </c>
-      <c r="P11" s="1" t="s">
+      <c r="Q11" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="Q11" s="1" t="s">
+      <c r="R11" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R11" s="3">
+      <c r="S11" s="11">
         <v>2311580115485</v>
       </c>
-      <c r="AK11" s="1" t="s">
+      <c r="AL11" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>sabbirahmed</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F12" s="1">
+      <c r="G12" s="9">
         <v>1937600512</v>
       </c>
-      <c r="H12" s="1">
+      <c r="I12" s="9">
         <v>1935591796</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="J12" s="1">
+      <c r="K12" s="9">
         <v>8500</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="L12" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L12" s="2">
+      <c r="M12" s="10">
         <v>45976</v>
       </c>
-      <c r="M12" s="2"/>
-      <c r="N12" s="1" t="s">
+      <c r="N12" s="10"/>
+      <c r="O12" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O12" s="2">
+      <c r="P12" s="10">
         <v>38644</v>
       </c>
-      <c r="P12" s="1" t="s">
+      <c r="Q12" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="Q12" s="1" t="s">
+      <c r="R12" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R12" s="3">
+      <c r="S12" s="11">
         <v>1731580447892</v>
       </c>
-      <c r="AK12" s="1" t="s">
+      <c r="AL12" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>hasanmia</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="1">
+      <c r="G13" s="9">
         <v>1984217911</v>
       </c>
-      <c r="G13" s="1">
+      <c r="H13" s="9">
         <v>1775222954</v>
       </c>
-      <c r="H13" s="1">
+      <c r="I13" s="9">
         <v>1935591918</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="J13" s="1">
+      <c r="K13" s="9">
         <v>8500</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L13" s="2">
+      <c r="M13" s="10">
         <v>45909</v>
       </c>
-      <c r="M13" s="2"/>
-      <c r="N13" s="1" t="s">
+      <c r="N13" s="10"/>
+      <c r="O13" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O13" s="2">
+      <c r="P13" s="10">
         <v>35458</v>
       </c>
-      <c r="P13" s="1" t="s">
+      <c r="Q13" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="Q13" s="1" t="s">
+      <c r="R13" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R13" s="3">
+      <c r="S13" s="11">
         <v>2311030047576</v>
       </c>
-      <c r="AK13" s="1" t="s">
+      <c r="AL13" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="1">
+      <c r="G14" s="9">
         <v>1984217912</v>
       </c>
-      <c r="H14" s="1">
+      <c r="I14" s="9">
         <v>1935591999</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="J14" s="1">
+      <c r="K14" s="9">
         <v>8500</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L14" s="2">
+      <c r="M14" s="10">
         <v>45965</v>
       </c>
-      <c r="M14" s="2"/>
-      <c r="N14" s="1" t="s">
+      <c r="N14" s="10"/>
+      <c r="O14" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O14" s="2">
+      <c r="P14" s="10">
         <v>38845</v>
       </c>
-      <c r="P14" s="1" t="s">
+      <c r="Q14" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="Q14" s="1" t="s">
+      <c r="R14" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R14" s="3">
+      <c r="S14" s="11">
         <v>2311030422596</v>
       </c>
-      <c r="AK14" s="1" t="s">
+      <c r="AL14" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>mahmudhasan</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="1">
+      <c r="G15" s="9">
         <v>1984220363</v>
       </c>
-      <c r="G15" s="1">
+      <c r="H15" s="9">
         <v>1620502971</v>
       </c>
-      <c r="H15" s="1">
+      <c r="I15" s="9">
         <v>1935591917</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J15" s="1">
+      <c r="K15" s="9">
         <v>8500</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="L15" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L15" s="2">
+      <c r="M15" s="10">
         <v>45748</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="1" t="s">
+      <c r="N15" s="10"/>
+      <c r="O15" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O15" s="2">
+      <c r="P15" s="10">
         <v>33898</v>
       </c>
-      <c r="P15" s="1" t="s">
+      <c r="Q15" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="Q15" s="1" t="s">
+      <c r="R15" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R15" s="3">
+      <c r="S15" s="11">
         <v>1731580062730</v>
       </c>
-      <c r="AK15" s="1" t="s">
+      <c r="AL15" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>ferozmia</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="1">
+      <c r="G16" s="9">
         <v>1984220364</v>
       </c>
-      <c r="G16" s="1">
+      <c r="H16" s="9">
         <v>1997616187</v>
       </c>
-      <c r="H16" s="1">
+      <c r="I16" s="9">
         <v>1935591855</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J16" s="1">
+      <c r="K16" s="9">
         <v>8500</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="L16" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L16" s="2">
+      <c r="M16" s="10">
         <v>45999</v>
       </c>
-      <c r="M16" s="2"/>
-      <c r="N16" s="1" t="s">
+      <c r="N16" s="10"/>
+      <c r="O16" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O16" s="2">
+      <c r="P16" s="10">
         <v>37991</v>
       </c>
-      <c r="P16" s="1" t="s">
+      <c r="Q16" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="Q16" s="1" t="s">
+      <c r="R16" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R16" s="3">
+      <c r="S16" s="11">
         <v>1737348886514</v>
       </c>
-      <c r="AK16" s="1" t="s">
+      <c r="AL16" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>hridoymia365</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F17" s="1">
+      <c r="G17" s="9">
         <v>1984220365</v>
       </c>
-      <c r="G17" s="1">
+      <c r="H17" s="9">
         <v>1970772132</v>
       </c>
-      <c r="H17" s="1">
+      <c r="I17" s="9">
         <v>1935591913</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J17" s="1">
+      <c r="K17" s="9">
         <v>8404</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="L17" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L17" s="2">
+      <c r="M17" s="10">
         <v>43709</v>
       </c>
-      <c r="M17" s="2"/>
-      <c r="N17" s="1" t="s">
+      <c r="N17" s="10"/>
+      <c r="O17" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O17" s="2">
+      <c r="P17" s="10">
         <v>36114</v>
       </c>
-      <c r="P17" s="1" t="s">
+      <c r="Q17" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="Q17" s="1" t="s">
+      <c r="R17" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R17" s="3">
+      <c r="S17" s="11">
         <v>1731030011132</v>
       </c>
-      <c r="AK17" s="1" t="s">
+      <c r="AL17" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>hridoymia366</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="1">
+      <c r="G18" s="9">
         <v>1984220366</v>
       </c>
-      <c r="G18" s="1">
+      <c r="H18" s="9">
         <v>1915343494</v>
       </c>
-      <c r="H18" s="1">
+      <c r="I18" s="9">
         <v>1935592054</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J18" s="1">
+      <c r="K18" s="9">
         <v>8580</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L18" s="2">
+      <c r="M18" s="10">
         <v>44470</v>
       </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="1" t="s">
+      <c r="N18" s="10"/>
+      <c r="O18" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O18" s="2">
+      <c r="P18" s="10">
         <v>36318</v>
       </c>
-      <c r="P18" s="1" t="s">
+      <c r="Q18" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="Q18" s="1" t="s">
+      <c r="R18" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R18" s="3">
+      <c r="S18" s="11">
         <v>1731510173296</v>
       </c>
-      <c r="AK18" s="1" t="s">
+      <c r="AL18" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F19" s="1">
+      <c r="G19" s="9">
         <v>1986646474</v>
       </c>
-      <c r="H19" s="1">
+      <c r="I19" s="9">
         <v>1935592053</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J19" s="1">
+      <c r="K19" s="9">
         <v>9350</v>
       </c>
-      <c r="K19" s="1" t="s">
+      <c r="L19" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L19" s="2">
+      <c r="M19" s="10">
         <v>45444</v>
       </c>
-      <c r="M19" s="2"/>
-      <c r="N19" s="1" t="s">
+      <c r="N19" s="10"/>
+      <c r="O19" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O19" s="2">
+      <c r="P19" s="10">
         <v>32174</v>
       </c>
-      <c r="P19" s="1" t="s">
+      <c r="Q19" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="Q19" s="1" t="s">
+      <c r="R19" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="R19" s="3">
+      <c r="S19" s="11">
         <v>7017332507958</v>
       </c>
-      <c r="AK19" s="1" t="s">
+      <c r="AL19" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="20" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>mijan</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F20" s="1">
+      <c r="G20" s="9">
         <v>1986686880</v>
       </c>
-      <c r="G20" s="4">
+      <c r="H20" s="12">
         <v>1924303333</v>
       </c>
-      <c r="H20" s="1">
+      <c r="I20" s="9">
         <v>1935591915</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="J20" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J20" s="1">
+      <c r="K20" s="9">
         <v>8500</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="L20" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L20" s="2">
+      <c r="M20" s="10">
         <v>46023</v>
       </c>
-      <c r="M20" s="2"/>
-      <c r="N20" s="1" t="s">
+      <c r="N20" s="10"/>
+      <c r="O20" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O20" s="2">
+      <c r="P20" s="10">
         <v>36557</v>
       </c>
-      <c r="P20" s="1" t="s">
+      <c r="Q20" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="Q20" s="1" t="s">
+      <c r="R20" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R20" s="3">
+      <c r="S20" s="11">
         <v>1731030011127</v>
       </c>
-      <c r="AK20" s="1" t="s">
+      <c r="AL20" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>toriqulislam</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G21" s="4">
+      <c r="H21" s="12">
         <v>1912317878</v>
       </c>
-      <c r="H21" s="1">
+      <c r="I21" s="9">
         <v>1958041930</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="L21" s="2">
+      <c r="M21" s="10">
         <v>42370</v>
       </c>
-      <c r="M21" s="2"/>
-      <c r="N21" s="1" t="s">
+      <c r="N21" s="10"/>
+      <c r="O21" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O21" s="2">
+      <c r="P21" s="10">
         <v>33675</v>
       </c>
-      <c r="P21" s="1" t="s">
+      <c r="Q21" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="Q21" s="1" t="s">
+      <c r="R21" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R21" s="3">
+      <c r="S21" s="11">
         <v>1731510105407</v>
       </c>
     </row>
-    <row r="22" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="9" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>sherali</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G22" s="4">
+      <c r="H22" s="12">
         <v>1911626293</v>
       </c>
-      <c r="H22" s="1">
+      <c r="I22" s="9">
         <v>1958041928</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="J22" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="L22" s="2">
+      <c r="M22" s="10">
         <v>41122</v>
       </c>
-      <c r="M22" s="2"/>
-      <c r="N22" s="1" t="s">
+      <c r="N22" s="10"/>
+      <c r="O22" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O22" s="2">
+      <c r="P22" s="10">
         <v>30806</v>
       </c>
-      <c r="P22" s="1" t="s">
+      <c r="Q22" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="Q22" s="1" t="s">
+      <c r="R22" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R22" s="3">
+      <c r="S22" s="11">
         <v>1471030170630</v>
       </c>
     </row>
-    <row r="23" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="C23" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G23" s="4">
+      <c r="H23" s="12">
         <v>1711228193</v>
       </c>
-      <c r="H23" s="1">
+      <c r="I23" s="9">
         <v>1935597976</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="J23" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="L23" s="2">
+      <c r="M23" s="10">
         <v>45870</v>
       </c>
-      <c r="M23" s="2"/>
-      <c r="N23" s="1" t="s">
+      <c r="N23" s="10"/>
+      <c r="O23" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O23" s="2">
+      <c r="P23" s="10">
         <v>30806</v>
       </c>
-      <c r="P23" s="7">
+      <c r="Q23" s="9">
         <v>2860896055</v>
       </c>
-      <c r="Q23" s="1" t="s">
+      <c r="R23" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R23" s="3">
+      <c r="S23" s="11">
         <v>1731030011382</v>
       </c>
     </row>
-    <row r="24" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+    <row r="24" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="D24" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G24" s="1">
+      <c r="H24" s="9">
         <v>1913453027</v>
       </c>
-      <c r="H24" s="1">
+      <c r="I24" s="9">
         <v>1935597774</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="J24" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="L24" s="2">
+      <c r="M24" s="10">
         <v>46054</v>
       </c>
-      <c r="M24" s="2"/>
-      <c r="N24" s="1" t="s">
+      <c r="N24" s="10"/>
+      <c r="O24" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O24" s="2">
+      <c r="P24" s="10">
         <v>37337</v>
       </c>
-      <c r="P24" s="1" t="s">
+      <c r="Q24" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="Q24" s="1" t="s">
+      <c r="R24" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R24" s="3">
+      <c r="S24" s="11">
         <v>1731050036178</v>
       </c>
     </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="C25" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="D25" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="E25" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="F25" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G25" s="13">
+      <c r="H25" s="5">
         <v>1786080093</v>
       </c>
-      <c r="H25" s="13">
+      <c r="I25" s="5">
         <v>1410678746</v>
       </c>
-      <c r="I25" s="13" t="s">
+      <c r="J25" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="J25" s="13">
+      <c r="K25" s="5">
         <v>10000</v>
       </c>
-      <c r="L25" s="14">
+      <c r="M25" s="6">
         <v>46082</v>
       </c>
-      <c r="N25" s="13" t="s">
+      <c r="O25" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O25" s="14">
+      <c r="P25" s="6">
         <v>33834</v>
       </c>
-      <c r="P25" s="15">
+      <c r="Q25" s="7">
         <v>6404733260</v>
       </c>
-      <c r="Q25" s="13" t="s">
+      <c r="R25" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R25" s="15">
+      <c r="S25" s="7">
         <v>1731580493357</v>
       </c>
-      <c r="V25" s="13" t="s">
+      <c r="W25" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="W25" s="13">
+      <c r="X25" s="5">
         <v>1752787879</v>
       </c>
-      <c r="X25" s="13" t="s">
+      <c r="Y25" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="Z25" s="13" t="s">
+      <c r="AA25" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="AA25" s="13" t="s">
+      <c r="AB25" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB25" s="13" t="s">
+      <c r="AC25" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="AC25" s="13" t="s">
+      <c r="AD25" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="AD25" s="13" t="s">
+      <c r="AE25" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="AE25" s="13" t="s">
+      <c r="AF25" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="AF25" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG25" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH25" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI25" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ25" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK25" s="13" t="s">
+      <c r="AG25" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH25" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI25" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ25" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK25" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL25" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="C26" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="D26" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="E26" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="F26" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G26" s="13">
+      <c r="H26" s="5">
         <v>1410071973</v>
       </c>
-      <c r="H26" s="13">
+      <c r="I26" s="5">
         <v>1410071973</v>
       </c>
-      <c r="I26" s="13" t="s">
+      <c r="J26" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="J26" s="13">
+      <c r="K26" s="5">
         <v>10000</v>
       </c>
-      <c r="L26" s="14">
+      <c r="M26" s="6">
         <v>46082</v>
       </c>
-      <c r="N26" s="13" t="s">
+      <c r="O26" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O26" s="14">
+      <c r="P26" s="6">
         <v>32540</v>
       </c>
-      <c r="P26" s="15">
+      <c r="Q26" s="7">
         <v>1314935507162</v>
       </c>
-      <c r="Q26" s="13" t="s">
+      <c r="R26" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R26" s="15">
+      <c r="S26" s="7">
         <v>1731580492738</v>
       </c>
-      <c r="S26" s="13" t="s">
+      <c r="T26" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="V26" s="13" t="s">
+      <c r="W26" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="W26" s="13">
+      <c r="X26" s="5">
         <v>1864929394</v>
       </c>
-      <c r="X26" s="13" t="s">
+      <c r="Y26" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="Z26" s="13" t="s">
+      <c r="AA26" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="AA26" s="13" t="s">
+      <c r="AB26" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB26" s="13" t="s">
+      <c r="AC26" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="AC26" s="13" t="s">
+      <c r="AD26" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="AD26" s="13" t="s">
+      <c r="AE26" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="AE26" s="13" t="s">
+      <c r="AF26" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="AF26" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG26" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH26" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI26" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ26" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK26" s="13" t="s">
+      <c r="AG26" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH26" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI26" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ26" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK26" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL26" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+    <row r="27" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="5" t="str">
+        <f>VLOOKUP($E:$E,[1]Sheet1!$B:$C,2,0)</f>
+        <v>shuvo</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="D27" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="E27" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="F27" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G27" s="13">
+      <c r="H27" s="5">
         <v>1410240211</v>
       </c>
-      <c r="H27" s="13">
+      <c r="I27" s="5">
         <v>1410240211</v>
       </c>
-      <c r="I27" s="13" t="s">
+      <c r="J27" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="J27" s="13">
+      <c r="K27" s="5">
         <v>10000</v>
       </c>
-      <c r="L27" s="14">
+      <c r="M27" s="6">
         <v>45971</v>
       </c>
-      <c r="N27" s="13" t="s">
+      <c r="O27" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O27" s="14">
+      <c r="P27" s="6">
         <v>1</v>
       </c>
-      <c r="P27" s="15">
+      <c r="Q27" s="7">
         <v>2863545949</v>
       </c>
-      <c r="Q27" s="13" t="s">
+      <c r="R27" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R27" s="15">
+      <c r="S27" s="7">
         <v>1731050292189</v>
       </c>
-      <c r="V27" s="13" t="s">
+      <c r="W27" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="W27" s="13">
+      <c r="X27" s="5">
         <v>1407911493</v>
       </c>
-      <c r="X27" s="13" t="s">
+      <c r="Y27" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="Z27" s="13" t="s">
+      <c r="AA27" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="AA27" s="13" t="s">
+      <c r="AB27" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB27" s="13" t="s">
+      <c r="AC27" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="AC27" s="13" t="s">
+      <c r="AD27" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="AD27" s="13" t="s">
+      <c r="AE27" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="AE27" s="13" t="s">
+      <c r="AF27" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="AF27" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG27" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH27" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI27" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ27" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK27" s="13" t="s">
+      <c r="AG27" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH27" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI27" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ27" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK27" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL27" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+    <row r="28" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="C28" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="D28" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="E28" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="F28" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G28" s="13">
+      <c r="H28" s="5">
         <v>1917787990</v>
       </c>
-      <c r="H28" s="13">
+      <c r="I28" s="5">
         <v>1410436602</v>
       </c>
-      <c r="I28" s="13" t="s">
+      <c r="J28" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="J28" s="13">
+      <c r="K28" s="5">
         <v>10000</v>
       </c>
-      <c r="L28" s="14">
+      <c r="M28" s="6">
         <v>45971</v>
       </c>
-      <c r="N28" s="13" t="s">
+      <c r="O28" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O28" s="14">
+      <c r="P28" s="6">
         <v>31595</v>
       </c>
-      <c r="P28" s="15">
+      <c r="Q28" s="7">
         <v>4813347971938</v>
       </c>
-      <c r="Q28" s="13" t="s">
+      <c r="R28" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R28" s="15">
+      <c r="S28" s="7">
         <v>2311580489016</v>
       </c>
-      <c r="V28" s="13" t="s">
+      <c r="W28" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="W28" s="13">
+      <c r="X28" s="5">
         <v>1730797404</v>
       </c>
-      <c r="X28" s="13" t="s">
+      <c r="Y28" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="Z28" s="13" t="s">
+      <c r="AA28" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="AA28" s="13" t="s">
+      <c r="AB28" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB28" s="13" t="s">
+      <c r="AC28" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="AC28" s="13" t="s">
+      <c r="AD28" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="AD28" s="13" t="s">
+      <c r="AE28" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="AE28" s="13" t="s">
+      <c r="AF28" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="AF28" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG28" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH28" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI28" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ28" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK28" s="13" t="s">
+      <c r="AG28" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH28" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI28" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ28" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK28" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL28" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="C29" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="D29" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="E29" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="F29" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G29" s="13">
+      <c r="H29" s="5">
         <v>1305213723</v>
       </c>
-      <c r="H29" s="13">
+      <c r="I29" s="5">
         <v>1410213723</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="J29" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="J29" s="13">
+      <c r="K29" s="5">
         <v>10000</v>
       </c>
-      <c r="L29" s="14">
+      <c r="M29" s="6">
         <v>46054</v>
       </c>
-      <c r="N29" s="13" t="s">
+      <c r="O29" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O29" s="14">
+      <c r="P29" s="6">
         <v>38161</v>
       </c>
-      <c r="P29" s="15">
+      <c r="Q29" s="7">
         <v>1042040244</v>
       </c>
-      <c r="Q29" s="13" t="s">
+      <c r="R29" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R29" s="15">
+      <c r="S29" s="7">
         <v>2311580512005</v>
       </c>
-      <c r="V29" s="13" t="s">
+      <c r="W29" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="W29" s="13">
+      <c r="X29" s="5">
         <v>1782371767</v>
       </c>
-      <c r="X29" s="13" t="s">
+      <c r="Y29" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="Z29" s="13" t="s">
+      <c r="AA29" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="AA29" s="13" t="s">
+      <c r="AB29" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB29" s="13" t="s">
+      <c r="AC29" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="AC29" s="13" t="s">
+      <c r="AD29" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="AD29" s="13" t="s">
+      <c r="AE29" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="AE29" s="13" t="s">
+      <c r="AF29" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="AF29" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG29" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH29" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI29" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ29" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK29" s="13" t="s">
+      <c r="AG29" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH29" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI29" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ29" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK29" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL29" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
+    <row r="30" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="C30" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="D30" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="E30" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="F30" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G30" s="13">
+      <c r="H30" s="5">
         <v>1990757830</v>
       </c>
-      <c r="H30" s="13">
+      <c r="I30" s="5">
         <v>1410173774</v>
       </c>
-      <c r="I30" s="13" t="s">
+      <c r="J30" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="J30" s="13">
+      <c r="K30" s="5">
         <v>10000</v>
       </c>
-      <c r="L30" s="14">
+      <c r="M30" s="6">
         <v>46054</v>
       </c>
-      <c r="N30" s="13" t="s">
+      <c r="O30" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O30" s="14">
+      <c r="P30" s="6">
         <v>33970</v>
       </c>
-      <c r="P30" s="15">
+      <c r="Q30" s="7">
         <v>2824445262</v>
       </c>
-      <c r="Q30" s="13" t="s">
+      <c r="R30" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="R30" s="15">
+      <c r="S30" s="7">
         <v>7017344002631</v>
       </c>
-      <c r="V30" s="13" t="s">
+      <c r="W30" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="W30" s="13">
+      <c r="X30" s="5">
         <v>1925717710</v>
       </c>
-      <c r="X30" s="13" t="s">
+      <c r="Y30" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="Z30" s="13" t="s">
+      <c r="AA30" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="AA30" s="13" t="s">
+      <c r="AB30" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB30" s="13" t="s">
+      <c r="AC30" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="AC30" s="13" t="s">
+      <c r="AD30" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="AD30" s="13" t="s">
+      <c r="AE30" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="AE30" s="13" t="s">
+      <c r="AF30" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="AF30" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG30" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH30" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI30" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ30" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK30" s="13" t="s">
+      <c r="AG30" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH30" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI30" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ30" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK30" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL30" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+    <row r="31" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="C31" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="E31" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="F31" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G31" s="13">
+      <c r="H31" s="5">
         <v>1763122889</v>
       </c>
-      <c r="H31" s="13">
+      <c r="I31" s="5">
         <v>1410720313</v>
       </c>
-      <c r="I31" s="13" t="s">
+      <c r="J31" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="J31" s="13">
+      <c r="K31" s="5">
         <v>10000</v>
       </c>
-      <c r="L31" s="14">
+      <c r="M31" s="6">
         <v>46143</v>
       </c>
-      <c r="N31" s="13" t="s">
+      <c r="O31" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O31" s="14">
+      <c r="P31" s="6">
         <v>36906</v>
       </c>
-      <c r="P31" s="15">
+      <c r="Q31" s="7">
         <v>8263476999</v>
       </c>
-      <c r="Q31" s="13" t="s">
+      <c r="R31" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R31" s="15">
+      <c r="S31" s="7">
         <v>1731580441218</v>
       </c>
-      <c r="S31" s="13" t="s">
+      <c r="T31" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="T31" s="13" t="s">
+      <c r="U31" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="U31" s="13" t="s">
+      <c r="V31" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="V31" s="13" t="s">
+      <c r="W31" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="W31" s="13">
+      <c r="X31" s="5">
         <v>1325533299</v>
       </c>
-      <c r="X31" s="13" t="s">
+      <c r="Y31" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="Y31" s="13" t="s">
+      <c r="Z31" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="Z31" s="13" t="s">
+      <c r="AA31" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="AA31" s="13" t="s">
+      <c r="AB31" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB31" s="13" t="s">
+      <c r="AC31" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="AC31" s="13" t="s">
+      <c r="AD31" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="AD31" s="13" t="s">
+      <c r="AE31" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="AE31" s="13" t="s">
+      <c r="AF31" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="AF31" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG31" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH31" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI31" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ31" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK31" s="13" t="s">
+      <c r="AG31" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH31" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI31" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ31" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK31" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL31" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
+    <row r="32" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="C32" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="E32" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="F32" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G32" s="13">
+      <c r="H32" s="5">
         <v>1984397910</v>
       </c>
-      <c r="H32" s="13">
+      <c r="I32" s="5">
         <v>1410031485</v>
       </c>
-      <c r="I32" s="13" t="s">
+      <c r="J32" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="J32" s="13">
+      <c r="K32" s="5">
         <v>10000</v>
       </c>
-      <c r="L32" s="14">
+      <c r="M32" s="6">
         <v>46143</v>
       </c>
-      <c r="N32" s="13" t="s">
+      <c r="O32" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O32" s="14">
+      <c r="P32" s="6">
         <v>31902</v>
       </c>
-      <c r="P32" s="15">
+      <c r="Q32" s="7">
         <v>5546839951</v>
       </c>
-      <c r="Q32" s="13" t="s">
+      <c r="R32" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R32" s="15">
+      <c r="S32" s="7">
         <v>1731580504974</v>
       </c>
-      <c r="S32" s="13" t="s">
+      <c r="T32" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="T32" s="13" t="s">
+      <c r="U32" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="U32" s="13" t="s">
+      <c r="V32" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="V32" s="13" t="s">
+      <c r="W32" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="W32" s="13">
+      <c r="X32" s="5">
         <v>1812206330</v>
       </c>
-      <c r="X32" s="13" t="s">
+      <c r="Y32" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="Y32" s="13" t="s">
+      <c r="Z32" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="Z32" s="13" t="s">
+      <c r="AA32" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="AA32" s="13" t="s">
+      <c r="AB32" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="AB32" s="13" t="s">
+      <c r="AC32" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="AC32" s="13" t="s">
+      <c r="AD32" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="AD32" s="13" t="s">
+      <c r="AE32" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="AE32" s="13" t="s">
+      <c r="AF32" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="AF32" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG32" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH32" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI32" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ32" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK32" s="13" t="s">
+      <c r="AG32" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH32" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI32" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ32" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK32" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL32" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
+    <row r="33" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="C33" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="E33" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="E33" s="13" t="s">
+      <c r="F33" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="G33" s="13">
+      <c r="H33" s="5">
         <v>1319047328</v>
       </c>
-      <c r="H33" s="13">
+      <c r="I33" s="5">
         <v>1410284216</v>
       </c>
-      <c r="I33" s="13" t="s">
+      <c r="J33" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="J33" s="13">
+      <c r="K33" s="5">
         <v>10000</v>
       </c>
-      <c r="L33" s="14">
+      <c r="M33" s="6">
         <v>46153</v>
       </c>
-      <c r="N33" s="13" t="s">
+      <c r="O33" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O33" s="14">
+      <c r="P33" s="6">
         <v>36835</v>
       </c>
-      <c r="P33" s="15">
+      <c r="Q33" s="7">
         <v>5579571190</v>
       </c>
-      <c r="Q33" s="13" t="s">
+      <c r="R33" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="R33" s="15">
+      <c r="S33" s="7">
         <v>1731580505955</v>
       </c>
-      <c r="S33" s="13" t="s">
+      <c r="T33" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="T33" s="13" t="s">
+      <c r="U33" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="U33" s="13" t="s">
+      <c r="V33" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="V33" s="13" t="s">
+      <c r="W33" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="W33" s="13">
+      <c r="X33" s="5">
         <v>1834674262</v>
       </c>
-      <c r="X33" s="13" t="s">
+      <c r="Y33" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="Y33" s="13" t="s">
+      <c r="Z33" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="Z33" s="13" t="s">
+      <c r="AA33" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="AA33" s="13" t="s">
+      <c r="AB33" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB33" s="13" t="s">
+      <c r="AC33" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="AC33" s="13" t="s">
+      <c r="AD33" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="AD33" s="13" t="s">
+      <c r="AE33" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="AE33" s="13" t="s">
+      <c r="AF33" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="AF33" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG33" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH33" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI33" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ33" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK33" s="13" t="s">
+      <c r="AG33" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH33" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI33" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ33" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK33" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL33" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
+    <row r="34" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="C34" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="D34" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="E34" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="E34" s="16" t="s">
+      <c r="F34" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="G34" s="13">
+      <c r="H34" s="5">
         <v>1918580928</v>
       </c>
-      <c r="H34" s="13">
+      <c r="I34" s="5">
         <v>1918580928</v>
       </c>
-      <c r="L34" s="14">
+      <c r="M34" s="6">
         <v>45972</v>
       </c>
-      <c r="N34" s="13" t="s">
+      <c r="O34" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="O34" s="14">
+      <c r="P34" s="6">
         <v>30051</v>
       </c>
-      <c r="P34" s="15">
+      <c r="Q34" s="7">
         <v>4813347974417</v>
       </c>
-      <c r="Q34" s="13" t="s">
+      <c r="R34" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="R34" s="15">
+      <c r="S34" s="7">
         <v>7017017975193</v>
       </c>
-      <c r="V34" s="13" t="s">
+      <c r="W34" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="W34" s="13">
+      <c r="X34" s="5">
         <v>1712436301</v>
       </c>
-      <c r="X34" s="13" t="s">
+      <c r="Y34" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="Z34" s="13" t="s">
+      <c r="AA34" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="AA34" s="13" t="s">
+      <c r="AB34" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="AB34" s="13" t="s">
+      <c r="AC34" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="AC34" s="13" t="s">
+      <c r="AD34" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="AD34" s="13" t="s">
+      <c r="AE34" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="AE34" s="13" t="s">
+      <c r="AF34" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="AF34" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AG34" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AH34" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AI34" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ34" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK34" s="13" t="s">
+      <c r="AG34" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AH34" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AI34" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ34" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AK34" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL34" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="C35" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="E35" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F35" s="1">
+      <c r="G35" s="9">
         <v>1409944002</v>
       </c>
-      <c r="H35" s="1">
+      <c r="I35" s="9">
         <v>1935593313</v>
       </c>
-      <c r="I35" s="1" t="s">
+      <c r="J35" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="J35" s="1">
+      <c r="K35" s="9">
         <v>10000</v>
       </c>
-      <c r="K35" s="1" t="s">
+      <c r="L35" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="L35" s="1">
+      <c r="M35" s="9">
         <v>46100</v>
       </c>
-      <c r="M35" s="2"/>
-      <c r="N35" s="1" t="s">
+      <c r="N35" s="10"/>
+      <c r="O35" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O35" s="1">
+      <c r="P35" s="9">
         <v>38153</v>
       </c>
-      <c r="P35" s="1" t="s">
+      <c r="Q35" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="Q35" s="1" t="s">
+      <c r="R35" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R35" s="1">
+      <c r="S35" s="9">
         <v>2311580180685</v>
       </c>
-      <c r="AK35" s="1" t="s">
+      <c r="AL35" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="C36" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="E36" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="F36" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F36" s="1">
+      <c r="G36" s="9">
         <v>1915270104</v>
       </c>
-      <c r="H36" s="1">
+      <c r="I36" s="9">
         <v>1935591816</v>
       </c>
-      <c r="I36" s="1" t="s">
+      <c r="J36" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="J36" s="1">
+      <c r="K36" s="9">
         <v>7000</v>
       </c>
-      <c r="K36" s="1" t="s">
+      <c r="L36" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="L36" s="1">
+      <c r="M36" s="9">
         <v>45474</v>
       </c>
-      <c r="M36" s="2"/>
-      <c r="N36" s="1" t="s">
+      <c r="N36" s="10"/>
+      <c r="O36" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O36" s="1">
+      <c r="P36" s="9">
         <v>38443</v>
       </c>
-      <c r="P36" s="1" t="s">
+      <c r="Q36" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="Q36" s="1" t="s">
+      <c r="R36" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R36" s="1">
+      <c r="S36" s="9">
         <v>2311580121330</v>
       </c>
-      <c r="AK36" s="1" t="s">
+      <c r="AL36" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="C37" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="D37" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="F37" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F37" s="1">
+      <c r="G37" s="9">
         <v>1915270105</v>
       </c>
-      <c r="H37" s="1">
+      <c r="I37" s="9">
         <v>1935591916</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="J37" s="1">
+      <c r="K37" s="9">
         <v>9500</v>
       </c>
-      <c r="K37" s="1" t="s">
+      <c r="L37" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="L37" s="1">
+      <c r="M37" s="9">
         <v>45909</v>
       </c>
-      <c r="M37" s="2"/>
-      <c r="N37" s="1" t="s">
+      <c r="N37" s="10"/>
+      <c r="O37" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O37" s="1">
+      <c r="P37" s="9">
         <v>38952</v>
       </c>
-      <c r="P37" s="1" t="s">
+      <c r="Q37" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="Q37" s="1" t="s">
+      <c r="R37" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R37" s="1">
+      <c r="S37" s="9">
         <v>2311580453888</v>
       </c>
-      <c r="AK37" s="1" t="s">
+      <c r="AL37" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="38" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="C38" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="D38" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="E38" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F38" s="1">
+      <c r="G38" s="9">
         <v>1967042950</v>
       </c>
-      <c r="H38" s="1">
+      <c r="I38" s="9">
         <v>1935592484</v>
       </c>
-      <c r="I38" s="1" t="s">
+      <c r="J38" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="J38" s="1">
+      <c r="K38" s="9">
         <v>9500</v>
       </c>
-      <c r="K38" s="1" t="s">
+      <c r="L38" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="L38" s="1">
+      <c r="M38" s="9">
         <v>45909</v>
       </c>
-      <c r="M38" s="2"/>
-      <c r="N38" s="1" t="s">
+      <c r="N38" s="10"/>
+      <c r="O38" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O38" s="1">
+      <c r="P38" s="9">
         <v>38688</v>
       </c>
-      <c r="P38" s="1" t="s">
+      <c r="Q38" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="Q38" s="1" t="s">
+      <c r="R38" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R38" s="1">
+      <c r="S38" s="9">
         <v>2311030382527</v>
       </c>
-      <c r="AK38" s="1" t="s">
+      <c r="AL38" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="39" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="C39" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="D39" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="E39" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="F39" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F39" s="1">
+      <c r="G39" s="9">
         <v>1986686877</v>
       </c>
-      <c r="H39" s="1">
+      <c r="I39" s="9">
         <v>1935591836</v>
       </c>
-      <c r="I39" s="1" t="s">
+      <c r="J39" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="J39" s="1">
+      <c r="K39" s="9">
         <v>7000</v>
       </c>
-      <c r="K39" s="1" t="s">
+      <c r="L39" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="L39" s="1">
+      <c r="M39" s="9">
         <v>45658</v>
       </c>
-      <c r="M39" s="2"/>
-      <c r="N39" s="1" t="s">
+      <c r="N39" s="10"/>
+      <c r="O39" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O39" s="1">
+      <c r="P39" s="9">
         <v>37483</v>
       </c>
-      <c r="P39" s="1" t="s">
+      <c r="Q39" s="9" t="s">
         <v>282</v>
       </c>
-      <c r="Q39" s="1" t="s">
+      <c r="R39" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R39" s="1">
+      <c r="S39" s="9">
         <v>2311580181156</v>
       </c>
-      <c r="AK39" s="1" t="s">
+      <c r="AL39" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="40" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="D40" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="E40" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="F40" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F40" s="1">
+      <c r="G40" s="9">
         <v>1986686878</v>
       </c>
-      <c r="H40" s="1">
+      <c r="I40" s="9">
         <v>1935591828</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="9" t="s">
         <v>286</v>
       </c>
-      <c r="J40" s="1">
+      <c r="K40" s="9">
         <v>10500</v>
       </c>
-      <c r="K40" s="1" t="s">
+      <c r="L40" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="L40" s="1">
+      <c r="M40" s="9">
         <v>46027</v>
       </c>
-      <c r="M40" s="2"/>
-      <c r="N40" s="1" t="s">
+      <c r="N40" s="10"/>
+      <c r="O40" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O40" s="1">
+      <c r="P40" s="9">
         <v>35286</v>
       </c>
-      <c r="P40" s="1" t="s">
+      <c r="Q40" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="Q40" s="1" t="s">
+      <c r="R40" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R40" s="1">
+      <c r="S40" s="9">
         <v>1731030011244</v>
       </c>
-      <c r="AK40" s="1" t="s">
+      <c r="AL40" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="41" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
+    <row r="41" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="C41" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="D41" s="9" t="s">
         <v>289</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="E41" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F41" s="1">
+      <c r="G41" s="9">
         <v>1986686879</v>
       </c>
-      <c r="H41" s="1">
+      <c r="I41" s="9">
         <v>1935592119</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="J41" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="J41" s="1">
+      <c r="K41" s="9">
         <v>7500</v>
       </c>
-      <c r="K41" s="1" t="s">
+      <c r="L41" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="L41" s="1">
+      <c r="M41" s="9">
         <v>45292</v>
       </c>
-      <c r="M41" s="2"/>
-      <c r="N41" s="1" t="s">
+      <c r="N41" s="10"/>
+      <c r="O41" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="O41" s="1">
+      <c r="P41" s="9">
         <v>37244</v>
       </c>
-      <c r="P41" s="1" t="s">
+      <c r="Q41" s="9" t="s">
         <v>292</v>
       </c>
-      <c r="Q41" s="1" t="s">
+      <c r="R41" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R41" s="1">
+      <c r="S41" s="9">
         <v>2311580116900</v>
       </c>
-      <c r="AK41" s="1" t="s">
+      <c r="AL41" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="C42" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="E42" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="F42" s="9" t="s">
         <v>296</v>
       </c>
-      <c r="G42" s="1">
+      <c r="H42" s="9">
         <v>1611169592</v>
       </c>
-      <c r="H42" s="1">
+      <c r="I42" s="9">
         <v>1999968844</v>
       </c>
-      <c r="I42" s="1" t="s">
+      <c r="J42" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="L42" s="1">
+      <c r="M42" s="9">
         <v>45931</v>
       </c>
-      <c r="M42" s="2"/>
-      <c r="O42" s="1">
+      <c r="N42" s="10"/>
+      <c r="P42" s="9">
         <v>31821</v>
       </c>
-      <c r="P42" s="1" t="s">
+      <c r="Q42" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="Q42" s="1" t="s">
+      <c r="R42" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R42" s="1">
+      <c r="S42" s="9">
         <v>2311580467330</v>
       </c>
-      <c r="AK42" s="1" t="s">
+      <c r="AL42" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="43" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
+    <row r="43" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="C43" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="E43" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="9" t="s">
         <v>296</v>
       </c>
-      <c r="H43" s="1">
+      <c r="I43" s="9">
         <v>1935600928</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="9" t="s">
         <v>301</v>
       </c>
-      <c r="M43" s="2"/>
-      <c r="AK43" s="1" t="s">
+      <c r="N43" s="10"/>
+      <c r="AL43" s="9" t="s">
         <v>81</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="I1:I1048576">
+  <conditionalFormatting sqref="J1:J1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P1:P1048576">
+  <conditionalFormatting sqref="Q1:Q1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>